<commit_message>
revisio manual despres del merge
</commit_message>
<xml_diff>
--- a/docs/punts-mesura.xlsx
+++ b/docs/punts-mesura.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\sxs-impulsio\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\supersonic-at\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54445DE2-1441-4AF7-B417-8B7DBA88BF78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13A5D360-EFC0-4705-99B0-8BCB993DD464}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{4CA701B3-5EB8-45D8-B6BB-1F057196BE44}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="95">
   <si>
     <t>id</t>
   </si>
@@ -56,6 +56,27 @@
     <t>area</t>
   </si>
   <si>
+    <t>E-100</t>
+  </si>
+  <si>
+    <t>EI-100</t>
+  </si>
+  <si>
+    <t>EI-101</t>
+  </si>
+  <si>
+    <t>EI-102</t>
+  </si>
+  <si>
+    <t>E-150</t>
+  </si>
+  <si>
+    <t>ED-150</t>
+  </si>
+  <si>
+    <t>EI-150</t>
+  </si>
+  <si>
     <t>id_vell</t>
   </si>
   <si>
@@ -107,6 +128,168 @@
     <t>WT</t>
   </si>
   <si>
+    <t>PEC</t>
+  </si>
+  <si>
+    <t>EI101</t>
+  </si>
+  <si>
+    <t>EI102</t>
+  </si>
+  <si>
+    <t>ED150</t>
+  </si>
+  <si>
+    <t>EI150</t>
+  </si>
+  <si>
+    <t>E150</t>
+  </si>
+  <si>
+    <t>P200</t>
+  </si>
+  <si>
+    <t>P201</t>
+  </si>
+  <si>
+    <t>P202</t>
+  </si>
+  <si>
+    <t>PK202</t>
+  </si>
+  <si>
+    <t>PK201</t>
+  </si>
+  <si>
+    <t>P304</t>
+  </si>
+  <si>
+    <t>P303</t>
+  </si>
+  <si>
+    <t>SI5003</t>
+  </si>
+  <si>
+    <t>P300</t>
+  </si>
+  <si>
+    <t>PI304</t>
+  </si>
+  <si>
+    <t>PI303</t>
+  </si>
+  <si>
+    <t>P400</t>
+  </si>
+  <si>
+    <t>PR401</t>
+  </si>
+  <si>
+    <t>PI401A</t>
+  </si>
+  <si>
+    <t>PI402A</t>
+  </si>
+  <si>
+    <t>PR402</t>
+  </si>
+  <si>
+    <t>P600</t>
+  </si>
+  <si>
+    <t>PR601</t>
+  </si>
+  <si>
+    <t>PI601</t>
+  </si>
+  <si>
+    <t>EI733</t>
+  </si>
+  <si>
+    <t>ER750</t>
+  </si>
+  <si>
+    <t>ER770</t>
+  </si>
+  <si>
+    <t>EI7X2</t>
+  </si>
+  <si>
+    <t>EI772</t>
+  </si>
+  <si>
+    <t>EI752</t>
+  </si>
+  <si>
+    <t>E700</t>
+  </si>
+  <si>
+    <t>E800</t>
+  </si>
+  <si>
+    <t>EI806</t>
+  </si>
+  <si>
+    <t>EI801</t>
+  </si>
+  <si>
+    <t>EI-906</t>
+  </si>
+  <si>
+    <t>EI-9061006</t>
+  </si>
+  <si>
+    <t>EI-9001006</t>
+  </si>
+  <si>
+    <t>EI-1001</t>
+  </si>
+  <si>
+    <t>EI-901</t>
+  </si>
+  <si>
+    <t>EI-9001000</t>
+  </si>
+  <si>
+    <t>EI906</t>
+  </si>
+  <si>
+    <t>EI1006</t>
+  </si>
+  <si>
+    <t>Y100</t>
+  </si>
+  <si>
+    <t>Y120</t>
+  </si>
+  <si>
+    <t>Y160170</t>
+  </si>
+  <si>
+    <t>Y170</t>
+  </si>
+  <si>
+    <t>Y160</t>
+  </si>
+  <si>
+    <t>L650</t>
+  </si>
+  <si>
+    <t>LI651</t>
+  </si>
+  <si>
+    <t>LI660</t>
+  </si>
+  <si>
+    <t>L670</t>
+  </si>
+  <si>
+    <t>SB670</t>
+  </si>
+  <si>
+    <t>LI671</t>
+  </si>
+  <si>
     <t>id_letter</t>
   </si>
   <si>
@@ -119,20 +302,35 @@
     <t>BV</t>
   </si>
   <si>
-    <t>col</t>
-  </si>
-  <si>
-    <t>x</t>
-  </si>
-  <si>
-    <t>y</t>
+    <t>VI710</t>
+  </si>
+  <si>
+    <t>VR710</t>
+  </si>
+  <si>
+    <t>VI810</t>
+  </si>
+  <si>
+    <t>VR810</t>
+  </si>
+  <si>
+    <t>V700800</t>
+  </si>
+  <si>
+    <t>V700</t>
+  </si>
+  <si>
+    <t>V800</t>
+  </si>
+  <si>
+    <t>EI701</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -145,12 +343,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="7"/>
-      <color rgb="FF000000"/>
-      <name val="Consolas"/>
-      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -173,13 +365,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -515,7 +704,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80D9219E-119C-467C-9531-507D24E0A5C1}">
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:K71"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
@@ -528,21 +717,21 @@
     <col min="12" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>83</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>23</v>
+        <v>84</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>24</v>
+        <v>85</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>1</v>
@@ -551,42 +740,34 @@
         <v>2</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>26</v>
+        <v>86</v>
       </c>
       <c r="C2" s="1">
         <v>7</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="1" t="str">
+        <f>A2&amp;(B2+C2)</f>
+        <v>BV7</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="F2" s="1" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="H2" s="1">
         <v>350</v>
@@ -598,19 +779,13 @@
         <v>8</v>
       </c>
       <c r="K2" s="1">
-        <f t="shared" ref="K2:K8" si="0">PI()*(((I2-J2)*10^-3)^2/4)</f>
+        <f t="shared" ref="K2:K21" si="0">PI()*(((I2-J2)*10^-3)^2/4)</f>
         <v>9.4896329995100878E-2</v>
       </c>
-      <c r="L2" s="1">
-        <v>20</v>
-      </c>
-      <c r="M2" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>25</v>
+        <v>86</v>
       </c>
       <c r="B3" s="1">
         <v>104</v>
@@ -623,13 +798,13 @@
         <v>BV104-5</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="H3" s="1">
         <v>150</v>
@@ -644,16 +819,10 @@
         <f t="shared" si="0"/>
         <v>2.0995460053481439E-2</v>
       </c>
-      <c r="L3" s="1">
-        <v>10</v>
-      </c>
-      <c r="M3" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>25</v>
+        <v>86</v>
       </c>
       <c r="B4" s="1">
         <v>105</v>
@@ -666,13 +835,13 @@
         <v>BV105-1</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="H4" s="1">
         <v>150</v>
@@ -687,16 +856,10 @@
         <f t="shared" si="0"/>
         <v>2.0995460053481439E-2</v>
       </c>
-      <c r="L4" s="1">
-        <v>539</v>
-      </c>
-      <c r="M4" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>25</v>
+        <v>86</v>
       </c>
       <c r="B5" s="1">
         <v>106</v>
@@ -709,13 +872,13 @@
         <v>BV106-3</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="H5" s="1">
         <v>150</v>
@@ -730,16 +893,10 @@
         <f t="shared" si="0"/>
         <v>2.0995460053481439E-2</v>
       </c>
-      <c r="L5" s="1">
-        <v>537</v>
-      </c>
-      <c r="M5" s="1">
-        <v>821</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>25</v>
+        <v>86</v>
       </c>
       <c r="B6" s="1">
         <v>107</v>
@@ -752,13 +909,13 @@
         <v>BV107-2</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="H6" s="1">
         <v>150</v>
@@ -773,16 +930,10 @@
         <f t="shared" si="0"/>
         <v>2.0995460053481439E-2</v>
       </c>
-      <c r="L6" s="1">
-        <v>692</v>
-      </c>
-      <c r="M6" s="1">
-        <v>709</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>25</v>
+        <v>86</v>
       </c>
       <c r="B7" s="1">
         <v>108</v>
@@ -795,13 +946,13 @@
         <v>BV108-4</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="H7" s="1">
         <v>150</v>
@@ -816,16 +967,10 @@
         <f t="shared" si="0"/>
         <v>2.0995460053481439E-2</v>
       </c>
-      <c r="L7" s="1">
-        <v>766</v>
-      </c>
-      <c r="M7" s="1">
-        <v>770</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>25</v>
+        <v>86</v>
       </c>
       <c r="B8" s="1">
         <v>109</v>
@@ -838,13 +983,13 @@
         <v>BV109-6</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="H8" s="1">
         <v>150</v>
@@ -859,27 +1004,1839 @@
         <f t="shared" si="0"/>
         <v>3.116510177843532E-2</v>
       </c>
-      <c r="L8" s="1">
-        <v>694</v>
-      </c>
-      <c r="M8" s="1">
-        <v>829</v>
-      </c>
-    </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E17" s="2"/>
-    </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E18" s="2"/>
-    </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E19" s="2"/>
-    </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E20" s="2"/>
-    </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E21" s="2"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>1</v>
+      </c>
+      <c r="B9" s="1">
+        <v>100</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1</v>
+      </c>
+      <c r="D9" s="1" t="str">
+        <f>A9&amp;"-"&amp;(B9+C9)</f>
+        <v>1-101</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H9" s="1">
+        <v>200</v>
+      </c>
+      <c r="I9" s="1">
+        <v>220</v>
+      </c>
+      <c r="K9" s="1">
+        <f t="shared" si="0"/>
+        <v>3.8013271108436497E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>1</v>
+      </c>
+      <c r="B10" s="1">
+        <v>100</v>
+      </c>
+      <c r="C10" s="1">
+        <v>2</v>
+      </c>
+      <c r="D10" s="1" t="str">
+        <f t="shared" ref="D10:D69" si="2">A10&amp;"-"&amp;(B10+C10)</f>
+        <v>1-102</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H10" s="1">
+        <v>125</v>
+      </c>
+      <c r="I10" s="1">
+        <v>141</v>
+      </c>
+      <c r="K10" s="1">
+        <f t="shared" si="0"/>
+        <v>1.5614500886504672E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>1</v>
+      </c>
+      <c r="B11" s="1">
+        <v>100</v>
+      </c>
+      <c r="C11" s="1">
+        <v>3</v>
+      </c>
+      <c r="D11" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-103</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H11" s="1">
+        <v>80</v>
+      </c>
+      <c r="I11" s="1">
+        <v>88.9</v>
+      </c>
+      <c r="K11" s="1">
+        <f t="shared" si="0"/>
+        <v>6.2071666189443481E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>1</v>
+      </c>
+      <c r="B12" s="1">
+        <v>100</v>
+      </c>
+      <c r="C12" s="1">
+        <v>4</v>
+      </c>
+      <c r="D12" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-104</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H12" s="1">
+        <v>80</v>
+      </c>
+      <c r="I12" s="1">
+        <v>88.9</v>
+      </c>
+      <c r="K12" s="1">
+        <f t="shared" si="0"/>
+        <v>6.2071666189443481E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="1">
+        <v>1</v>
+      </c>
+      <c r="B13" s="1">
+        <v>100</v>
+      </c>
+      <c r="C13" s="1">
+        <v>5</v>
+      </c>
+      <c r="D13" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-105</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H13" s="1">
+        <v>200</v>
+      </c>
+      <c r="I13" s="1">
+        <v>220</v>
+      </c>
+      <c r="K13" s="1">
+        <f t="shared" si="0"/>
+        <v>3.8013271108436497E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" s="1">
+        <v>1</v>
+      </c>
+      <c r="B14" s="1">
+        <v>100</v>
+      </c>
+      <c r="C14" s="1">
+        <v>6</v>
+      </c>
+      <c r="D14" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-106</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H14" s="1">
+        <v>50</v>
+      </c>
+      <c r="I14" s="1">
+        <v>60.3</v>
+      </c>
+      <c r="K14" s="1">
+        <f t="shared" si="0"/>
+        <v>2.8557784079478277E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" s="1">
+        <v>1</v>
+      </c>
+      <c r="B15" s="1">
+        <v>100</v>
+      </c>
+      <c r="C15" s="1">
+        <v>7</v>
+      </c>
+      <c r="D15" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-107</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H15" s="1">
+        <v>50</v>
+      </c>
+      <c r="I15" s="1">
+        <v>60.3</v>
+      </c>
+      <c r="K15" s="1">
+        <f t="shared" si="0"/>
+        <v>2.8557784079478277E-3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" s="1">
+        <v>1</v>
+      </c>
+      <c r="B16" s="1">
+        <v>100</v>
+      </c>
+      <c r="C16" s="1">
+        <v>8</v>
+      </c>
+      <c r="D16" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-108</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H16" s="1">
+        <v>80</v>
+      </c>
+      <c r="I16" s="1">
+        <v>88.9</v>
+      </c>
+      <c r="K16" s="1">
+        <f t="shared" si="0"/>
+        <v>6.2071666189443481E-3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" s="1">
+        <v>6</v>
+      </c>
+      <c r="B17" s="1">
+        <v>100</v>
+      </c>
+      <c r="C17" s="1">
+        <v>1</v>
+      </c>
+      <c r="D17" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>6-101</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H17" s="1">
+        <v>204</v>
+      </c>
+      <c r="I17" s="1">
+        <v>204</v>
+      </c>
+      <c r="K17" s="1">
+        <f t="shared" si="0"/>
+        <v>3.2685129967948215E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18" s="1">
+        <v>6</v>
+      </c>
+      <c r="B18" s="1">
+        <v>100</v>
+      </c>
+      <c r="C18" s="1">
+        <v>2</v>
+      </c>
+      <c r="D18" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>6-102</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H18" s="1">
+        <v>204</v>
+      </c>
+      <c r="I18" s="1">
+        <v>204</v>
+      </c>
+      <c r="K18" s="1">
+        <f t="shared" si="0"/>
+        <v>3.2685129967948215E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" s="1">
+        <v>6</v>
+      </c>
+      <c r="B19" s="1">
+        <v>100</v>
+      </c>
+      <c r="C19" s="1">
+        <v>3</v>
+      </c>
+      <c r="D19" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>6-103</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="H19" s="1">
+        <v>100</v>
+      </c>
+      <c r="I19" s="1">
+        <v>114</v>
+      </c>
+      <c r="K19" s="1">
+        <f t="shared" si="0"/>
+        <v>1.0207034531513238E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20" s="1">
+        <v>6</v>
+      </c>
+      <c r="B20" s="1">
+        <v>100</v>
+      </c>
+      <c r="C20" s="1">
+        <v>4</v>
+      </c>
+      <c r="D20" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>6-104</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H20" s="1">
+        <v>129</v>
+      </c>
+      <c r="I20" s="1">
+        <v>129</v>
+      </c>
+      <c r="K20" s="1">
+        <f t="shared" si="0"/>
+        <v>1.3069810837096936E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21" s="1">
+        <v>6</v>
+      </c>
+      <c r="B21" s="1">
+        <v>100</v>
+      </c>
+      <c r="C21" s="1">
+        <v>5</v>
+      </c>
+      <c r="D21" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>6-105</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="H21" s="1">
+        <v>129</v>
+      </c>
+      <c r="I21" s="1">
+        <v>129</v>
+      </c>
+      <c r="K21" s="1">
+        <f t="shared" si="0"/>
+        <v>1.3069810837096936E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A22" s="1">
+        <v>3</v>
+      </c>
+      <c r="B22" s="1">
+        <v>200</v>
+      </c>
+      <c r="C22" s="1">
+        <v>1</v>
+      </c>
+      <c r="D22" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>3-201</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H22" s="1">
+        <v>100</v>
+      </c>
+      <c r="I22" s="1">
+        <v>114</v>
+      </c>
+      <c r="K22" s="1">
+        <f t="shared" ref="K22:K62" si="3">PI()*(((I22-J22)*10^-3)^2/4)</f>
+        <v>1.0207034531513238E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23" s="1">
+        <v>3</v>
+      </c>
+      <c r="B23" s="1">
+        <v>200</v>
+      </c>
+      <c r="C23" s="1">
+        <v>2</v>
+      </c>
+      <c r="D23" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>3-202</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H23" s="1">
+        <v>65</v>
+      </c>
+      <c r="I23" s="1">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="K23" s="1">
+        <f t="shared" si="3"/>
+        <v>4.5484056978489359E-3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24" s="1">
+        <v>3</v>
+      </c>
+      <c r="B24" s="1">
+        <v>200</v>
+      </c>
+      <c r="C24" s="1">
+        <v>3</v>
+      </c>
+      <c r="D24" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>3-203</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H24" s="1">
+        <v>65</v>
+      </c>
+      <c r="I24" s="1">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="K24" s="1">
+        <f t="shared" si="3"/>
+        <v>4.5484056978489359E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A25" s="1">
+        <v>3</v>
+      </c>
+      <c r="B25" s="1">
+        <v>300</v>
+      </c>
+      <c r="C25" s="1">
+        <v>1</v>
+      </c>
+      <c r="D25" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>3-301</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H25" s="1">
+        <v>65</v>
+      </c>
+      <c r="I25" s="1">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="K25" s="1">
+        <f t="shared" si="3"/>
+        <v>4.5484056978489359E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A26" s="1">
+        <v>3</v>
+      </c>
+      <c r="B26" s="1">
+        <v>300</v>
+      </c>
+      <c r="C26" s="1">
+        <v>2</v>
+      </c>
+      <c r="D26" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>3-302</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H26" s="1">
+        <v>50</v>
+      </c>
+      <c r="I26" s="1">
+        <v>60.3</v>
+      </c>
+      <c r="K26" s="1">
+        <f t="shared" si="3"/>
+        <v>2.8557784079478277E-3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A27" s="1">
+        <v>3</v>
+      </c>
+      <c r="B27" s="1">
+        <v>300</v>
+      </c>
+      <c r="C27" s="1">
+        <v>3</v>
+      </c>
+      <c r="D27" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>3-303</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H27" s="1">
+        <v>50</v>
+      </c>
+      <c r="I27" s="1">
+        <v>60.3</v>
+      </c>
+      <c r="K27" s="1">
+        <f t="shared" si="3"/>
+        <v>2.8557784079478277E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A28" s="1">
+        <v>3</v>
+      </c>
+      <c r="B28" s="1">
+        <v>300</v>
+      </c>
+      <c r="C28" s="1">
+        <v>4</v>
+      </c>
+      <c r="D28" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>3-304</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H28" s="1">
+        <v>32</v>
+      </c>
+      <c r="I28" s="1">
+        <v>42.2</v>
+      </c>
+      <c r="K28" s="1">
+        <f t="shared" si="3"/>
+        <v>1.3986684653047119E-3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A29" s="1">
+        <v>3</v>
+      </c>
+      <c r="B29" s="1">
+        <v>400</v>
+      </c>
+      <c r="C29" s="1">
+        <v>1</v>
+      </c>
+      <c r="D29" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>3-401</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H29" s="1">
+        <v>80</v>
+      </c>
+      <c r="I29" s="1">
+        <v>88.9</v>
+      </c>
+      <c r="K29" s="1">
+        <f t="shared" si="3"/>
+        <v>6.2071666189443481E-3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A30" s="1">
+        <v>3</v>
+      </c>
+      <c r="B30" s="1">
+        <v>400</v>
+      </c>
+      <c r="C30" s="1">
+        <v>2</v>
+      </c>
+      <c r="D30" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>3-402</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="H30" s="1">
+        <v>40</v>
+      </c>
+      <c r="I30" s="1">
+        <v>48.3</v>
+      </c>
+      <c r="K30" s="1">
+        <f t="shared" si="3"/>
+        <v>1.8322475214082729E-3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A31" s="1">
+        <v>3</v>
+      </c>
+      <c r="B31" s="1">
+        <v>400</v>
+      </c>
+      <c r="C31" s="1">
+        <v>3</v>
+      </c>
+      <c r="D31" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>3-403</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="H31" s="1">
+        <v>50</v>
+      </c>
+      <c r="I31" s="1">
+        <v>60.3</v>
+      </c>
+      <c r="K31" s="1">
+        <f t="shared" si="3"/>
+        <v>2.8557784079478277E-3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" s="1">
+        <v>3</v>
+      </c>
+      <c r="B32" s="1">
+        <v>400</v>
+      </c>
+      <c r="C32" s="1">
+        <v>4</v>
+      </c>
+      <c r="D32" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>3-404</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="H32" s="1">
+        <v>50</v>
+      </c>
+      <c r="I32" s="1">
+        <v>60.3</v>
+      </c>
+      <c r="K32" s="1">
+        <f t="shared" si="3"/>
+        <v>2.8557784079478277E-3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" s="1">
+        <v>3</v>
+      </c>
+      <c r="B33" s="1">
+        <v>400</v>
+      </c>
+      <c r="C33" s="1">
+        <v>5</v>
+      </c>
+      <c r="D33" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>3-405</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H33" s="1">
+        <v>40</v>
+      </c>
+      <c r="I33" s="1">
+        <v>48.3</v>
+      </c>
+      <c r="K33" s="1">
+        <f t="shared" si="3"/>
+        <v>1.8322475214082729E-3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A34" s="1">
+        <v>2</v>
+      </c>
+      <c r="B34" s="1">
+        <v>600</v>
+      </c>
+      <c r="C34" s="1">
+        <v>1</v>
+      </c>
+      <c r="D34" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>2-601</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H34" s="1">
+        <v>65</v>
+      </c>
+      <c r="I34" s="1">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="K34" s="1">
+        <f t="shared" si="3"/>
+        <v>4.5484056978489359E-3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35" s="1">
+        <v>2</v>
+      </c>
+      <c r="B35" s="1">
+        <v>600</v>
+      </c>
+      <c r="C35" s="1">
+        <v>2</v>
+      </c>
+      <c r="D35" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>2-602</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="H35" s="1">
+        <v>43</v>
+      </c>
+      <c r="I35" s="1">
+        <v>43</v>
+      </c>
+      <c r="K35" s="1">
+        <f t="shared" si="3"/>
+        <v>1.4522012041218821E-3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A36" s="1">
+        <v>2</v>
+      </c>
+      <c r="B36" s="1">
+        <v>600</v>
+      </c>
+      <c r="C36" s="1">
+        <v>3</v>
+      </c>
+      <c r="D36" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>2-603</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="H36" s="1">
+        <v>50</v>
+      </c>
+      <c r="I36" s="1">
+        <v>60.3</v>
+      </c>
+      <c r="K36" s="1">
+        <f t="shared" si="3"/>
+        <v>2.8557784079478277E-3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A37" s="1">
+        <v>2</v>
+      </c>
+      <c r="B37" s="1">
+        <v>600</v>
+      </c>
+      <c r="C37" s="1">
+        <v>4</v>
+      </c>
+      <c r="D37" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>2-604</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="H37" s="1">
+        <v>125</v>
+      </c>
+      <c r="I37" s="1">
+        <v>139</v>
+      </c>
+      <c r="K37" s="1">
+        <f t="shared" si="3"/>
+        <v>1.5174677915002103E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38" s="1">
+        <v>2</v>
+      </c>
+      <c r="B38" s="1">
+        <v>600</v>
+      </c>
+      <c r="C38" s="1">
+        <v>5</v>
+      </c>
+      <c r="D38" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>2-605</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="H38" s="1">
+        <v>100</v>
+      </c>
+      <c r="I38" s="1">
+        <v>114</v>
+      </c>
+      <c r="K38" s="1">
+        <f t="shared" si="3"/>
+        <v>1.0207034531513238E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39" s="1">
+        <v>2</v>
+      </c>
+      <c r="B39" s="1">
+        <v>600</v>
+      </c>
+      <c r="C39" s="1">
+        <v>6</v>
+      </c>
+      <c r="D39" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>2-606</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="H39" s="1">
+        <v>50</v>
+      </c>
+      <c r="I39" s="1">
+        <v>60.3</v>
+      </c>
+      <c r="K39" s="1">
+        <f t="shared" si="3"/>
+        <v>2.8557784079478277E-3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A40" s="1">
+        <v>3</v>
+      </c>
+      <c r="B40" s="1">
+        <v>600</v>
+      </c>
+      <c r="C40" s="1">
+        <v>1</v>
+      </c>
+      <c r="D40" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>3-601</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H40" s="1">
+        <v>50</v>
+      </c>
+      <c r="I40" s="1">
+        <v>60.3</v>
+      </c>
+      <c r="K40" s="1">
+        <f t="shared" si="3"/>
+        <v>2.8557784079478277E-3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41" s="1">
+        <v>3</v>
+      </c>
+      <c r="B41" s="1">
+        <v>600</v>
+      </c>
+      <c r="C41" s="1">
+        <v>2</v>
+      </c>
+      <c r="D41" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>3-602</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H41" s="1">
+        <v>50</v>
+      </c>
+      <c r="I41" s="1">
+        <v>60.3</v>
+      </c>
+      <c r="K41" s="1">
+        <f t="shared" si="3"/>
+        <v>2.8557784079478277E-3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42" s="1">
+        <v>3</v>
+      </c>
+      <c r="B42" s="1">
+        <v>600</v>
+      </c>
+      <c r="C42" s="1">
+        <v>3</v>
+      </c>
+      <c r="D42" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>3-603</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="H42" s="1">
+        <v>50</v>
+      </c>
+      <c r="I42" s="1">
+        <v>60.3</v>
+      </c>
+      <c r="K42" s="1">
+        <f>PI()*(((I42-J42)*10^-3)^2/4)</f>
+        <v>2.8557784079478277E-3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A43" s="1">
+        <v>1</v>
+      </c>
+      <c r="B43" s="1">
+        <v>700</v>
+      </c>
+      <c r="C43" s="1">
+        <v>1</v>
+      </c>
+      <c r="D43" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-701</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="H43" s="1">
+        <v>200</v>
+      </c>
+      <c r="I43" s="1">
+        <v>220</v>
+      </c>
+      <c r="K43" s="1">
+        <f t="shared" si="3"/>
+        <v>3.8013271108436497E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44" s="1">
+        <v>1</v>
+      </c>
+      <c r="B44" s="1">
+        <v>700</v>
+      </c>
+      <c r="C44" s="1">
+        <v>2</v>
+      </c>
+      <c r="D44" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-702</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="H44" s="1">
+        <v>80</v>
+      </c>
+      <c r="I44" s="1">
+        <v>88.9</v>
+      </c>
+      <c r="K44" s="1">
+        <f t="shared" si="3"/>
+        <v>6.2071666189443481E-3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45" s="1">
+        <v>1</v>
+      </c>
+      <c r="B45" s="1">
+        <v>700</v>
+      </c>
+      <c r="C45" s="1">
+        <v>3</v>
+      </c>
+      <c r="D45" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-703</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="K45" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46" s="1">
+        <v>1</v>
+      </c>
+      <c r="B46" s="1">
+        <v>700</v>
+      </c>
+      <c r="C46" s="1">
+        <v>4</v>
+      </c>
+      <c r="D46" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-704</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="K46" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47" s="1">
+        <v>1</v>
+      </c>
+      <c r="B47" s="1">
+        <v>700</v>
+      </c>
+      <c r="C47" s="1">
+        <v>5</v>
+      </c>
+      <c r="D47" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-705</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="H47" s="1">
+        <v>100</v>
+      </c>
+      <c r="I47" s="1">
+        <v>114</v>
+      </c>
+      <c r="K47" s="1">
+        <f t="shared" si="3"/>
+        <v>1.0207034531513238E-2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48" s="1">
+        <v>1</v>
+      </c>
+      <c r="B48" s="1">
+        <v>700</v>
+      </c>
+      <c r="C48" s="1">
+        <v>6</v>
+      </c>
+      <c r="D48" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-706</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H48" s="1">
+        <v>65</v>
+      </c>
+      <c r="I48" s="1">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="K48" s="1">
+        <f t="shared" si="3"/>
+        <v>4.5484056978489359E-3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A49" s="1">
+        <v>1</v>
+      </c>
+      <c r="B49" s="1">
+        <v>700</v>
+      </c>
+      <c r="C49" s="1">
+        <v>7</v>
+      </c>
+      <c r="D49" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-707</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="H49" s="1">
+        <v>80</v>
+      </c>
+      <c r="I49" s="1">
+        <v>88.9</v>
+      </c>
+      <c r="K49" s="1">
+        <f t="shared" si="3"/>
+        <v>6.2071666189443481E-3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A50" s="1">
+        <v>1</v>
+      </c>
+      <c r="B50" s="1">
+        <v>700</v>
+      </c>
+      <c r="C50" s="1">
+        <v>8</v>
+      </c>
+      <c r="D50" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-708</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H50" s="1">
+        <v>125</v>
+      </c>
+      <c r="I50" s="1">
+        <v>141</v>
+      </c>
+      <c r="K50" s="1">
+        <f t="shared" si="3"/>
+        <v>1.5614500886504672E-2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A51" s="1">
+        <v>1</v>
+      </c>
+      <c r="B51" s="1">
+        <v>800</v>
+      </c>
+      <c r="C51" s="1">
+        <v>1</v>
+      </c>
+      <c r="D51" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-801</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H51" s="1">
+        <v>155</v>
+      </c>
+      <c r="I51" s="1">
+        <v>155</v>
+      </c>
+      <c r="J51" s="1">
+        <v>1.8</v>
+      </c>
+      <c r="K51" s="1">
+        <f t="shared" si="3"/>
+        <v>1.8433483390497326E-2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A52" s="1">
+        <v>1</v>
+      </c>
+      <c r="B52" s="1">
+        <v>800</v>
+      </c>
+      <c r="C52" s="1">
+        <v>2</v>
+      </c>
+      <c r="D52" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-802</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H52" s="1">
+        <v>80</v>
+      </c>
+      <c r="I52" s="1">
+        <v>88.9</v>
+      </c>
+      <c r="K52" s="1">
+        <f t="shared" si="3"/>
+        <v>6.2071666189443481E-3</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A53" s="1">
+        <v>1</v>
+      </c>
+      <c r="B53" s="1">
+        <v>800</v>
+      </c>
+      <c r="C53" s="1">
+        <v>3</v>
+      </c>
+      <c r="D53" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-803</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H53" s="1">
+        <v>125</v>
+      </c>
+      <c r="I53" s="1">
+        <v>139.69999999999999</v>
+      </c>
+      <c r="K53" s="1">
+        <f t="shared" si="3"/>
+        <v>1.5327901242699303E-2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A54" s="1">
+        <v>1</v>
+      </c>
+      <c r="B54" s="1">
+        <v>900</v>
+      </c>
+      <c r="C54" s="1">
+        <v>1</v>
+      </c>
+      <c r="D54" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-901</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H54" s="1">
+        <v>204</v>
+      </c>
+      <c r="I54" s="1">
+        <v>204</v>
+      </c>
+      <c r="K54" s="1">
+        <f t="shared" si="3"/>
+        <v>3.2685129967948215E-2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A55" s="1">
+        <v>1</v>
+      </c>
+      <c r="B55" s="1">
+        <v>900</v>
+      </c>
+      <c r="C55" s="1">
+        <v>2</v>
+      </c>
+      <c r="D55" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-902</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="H55" s="1">
+        <v>204</v>
+      </c>
+      <c r="I55" s="1">
+        <v>204</v>
+      </c>
+      <c r="K55" s="1">
+        <f t="shared" si="3"/>
+        <v>3.2685129967948215E-2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A56" s="1">
+        <v>1</v>
+      </c>
+      <c r="B56" s="1">
+        <v>900</v>
+      </c>
+      <c r="C56" s="1">
+        <v>3</v>
+      </c>
+      <c r="D56" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-903</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H56" s="1">
+        <v>204</v>
+      </c>
+      <c r="I56" s="1">
+        <v>204</v>
+      </c>
+      <c r="K56" s="1">
+        <f t="shared" si="3"/>
+        <v>3.2685129967948215E-2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A57" s="1">
+        <v>1</v>
+      </c>
+      <c r="B57" s="1">
+        <v>900</v>
+      </c>
+      <c r="C57" s="1">
+        <v>4</v>
+      </c>
+      <c r="D57" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-904</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H57" s="1">
+        <v>155</v>
+      </c>
+      <c r="I57" s="1">
+        <v>154</v>
+      </c>
+      <c r="K57" s="1">
+        <f t="shared" si="3"/>
+        <v>1.8626502843133885E-2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A58" s="1">
+        <v>1</v>
+      </c>
+      <c r="B58" s="1">
+        <v>900</v>
+      </c>
+      <c r="C58" s="1">
+        <v>5</v>
+      </c>
+      <c r="D58" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-905</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H58" s="1">
+        <v>155</v>
+      </c>
+      <c r="I58" s="1">
+        <v>154</v>
+      </c>
+      <c r="K58" s="1">
+        <f t="shared" si="3"/>
+        <v>1.8626502843133885E-2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A59" s="1">
+        <v>1</v>
+      </c>
+      <c r="B59" s="1">
+        <v>900</v>
+      </c>
+      <c r="C59" s="1">
+        <v>6</v>
+      </c>
+      <c r="D59" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-906</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H59" s="1">
+        <v>80</v>
+      </c>
+      <c r="I59" s="1">
+        <v>88.9</v>
+      </c>
+      <c r="K59" s="1">
+        <f t="shared" si="3"/>
+        <v>6.2071666189443481E-3</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A60" s="1">
+        <v>1</v>
+      </c>
+      <c r="B60" s="1">
+        <v>900</v>
+      </c>
+      <c r="C60" s="1">
+        <v>7</v>
+      </c>
+      <c r="D60" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-907</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="H60" s="1">
+        <v>80</v>
+      </c>
+      <c r="I60" s="1">
+        <v>88.9</v>
+      </c>
+      <c r="K60" s="1">
+        <f t="shared" si="3"/>
+        <v>6.2071666189443481E-3</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A61" s="1">
+        <v>1</v>
+      </c>
+      <c r="B61" s="1">
+        <v>900</v>
+      </c>
+      <c r="C61" s="1">
+        <v>8</v>
+      </c>
+      <c r="D61" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-908</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H61" s="1">
+        <v>125</v>
+      </c>
+      <c r="I61" s="1">
+        <v>139.69999999999999</v>
+      </c>
+      <c r="K61" s="1">
+        <f t="shared" si="3"/>
+        <v>1.5327901242699303E-2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A62" s="1">
+        <v>1</v>
+      </c>
+      <c r="B62" s="1">
+        <v>900</v>
+      </c>
+      <c r="C62" s="1">
+        <v>9</v>
+      </c>
+      <c r="D62" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>1-909</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H62" s="1">
+        <v>125</v>
+      </c>
+      <c r="I62" s="1">
+        <v>139.69999999999999</v>
+      </c>
+      <c r="K62" s="1">
+        <f t="shared" si="3"/>
+        <v>1.5327901242699303E-2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A63" s="1">
+        <v>2</v>
+      </c>
+      <c r="B63" s="1">
+        <v>700</v>
+      </c>
+      <c r="C63" s="1">
+        <v>1</v>
+      </c>
+      <c r="D63" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>2-701</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H63" s="1">
+        <v>150</v>
+      </c>
+      <c r="I63" s="1">
+        <v>168.3</v>
+      </c>
+      <c r="K63" s="1">
+        <f t="shared" ref="K63:K69" si="4">PI()*(((I63-J63)*10^-3)^2/4)</f>
+        <v>2.2246316584434749E-2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A64" s="1">
+        <v>2</v>
+      </c>
+      <c r="B64" s="1">
+        <v>700</v>
+      </c>
+      <c r="C64" s="1">
+        <v>2</v>
+      </c>
+      <c r="D64" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>2-702</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H64" s="1">
+        <v>100</v>
+      </c>
+      <c r="I64" s="1">
+        <v>114</v>
+      </c>
+      <c r="K64" s="1">
+        <f t="shared" si="4"/>
+        <v>1.0207034531513238E-2</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A65" s="1">
+        <v>2</v>
+      </c>
+      <c r="B65" s="1">
+        <v>700</v>
+      </c>
+      <c r="C65" s="1">
+        <v>3</v>
+      </c>
+      <c r="D65" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>2-703</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H65" s="1">
+        <v>100</v>
+      </c>
+      <c r="I65" s="1">
+        <v>114</v>
+      </c>
+      <c r="K65" s="1">
+        <f t="shared" si="4"/>
+        <v>1.0207034531513238E-2</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A66" s="1">
+        <v>2</v>
+      </c>
+      <c r="B66" s="1">
+        <v>700</v>
+      </c>
+      <c r="C66" s="1">
+        <v>4</v>
+      </c>
+      <c r="D66" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>2-704</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="H66" s="1">
+        <v>65</v>
+      </c>
+      <c r="I66" s="1">
+        <v>73</v>
+      </c>
+      <c r="K66" s="1">
+        <f t="shared" si="4"/>
+        <v>4.1853868127450016E-3</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A67" s="1">
+        <v>2</v>
+      </c>
+      <c r="B67" s="1">
+        <v>700</v>
+      </c>
+      <c r="C67" s="1">
+        <v>5</v>
+      </c>
+      <c r="D67" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>2-705</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="H67" s="1">
+        <v>50</v>
+      </c>
+      <c r="I67" s="1">
+        <v>60.3</v>
+      </c>
+      <c r="K67" s="1">
+        <f t="shared" si="4"/>
+        <v>2.8557784079478277E-3</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A68" s="1">
+        <v>2</v>
+      </c>
+      <c r="B68" s="1">
+        <v>700</v>
+      </c>
+      <c r="C68" s="1">
+        <v>6</v>
+      </c>
+      <c r="D68" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>2-706</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H68" s="1">
+        <v>65</v>
+      </c>
+      <c r="I68" s="1">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="K68" s="1">
+        <f t="shared" si="4"/>
+        <v>4.5484056978489359E-3</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A69" s="1">
+        <v>2</v>
+      </c>
+      <c r="B69" s="1">
+        <v>700</v>
+      </c>
+      <c r="C69" s="1">
+        <v>7</v>
+      </c>
+      <c r="D69" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>2-707</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="H69" s="1">
+        <v>50</v>
+      </c>
+      <c r="I69" s="1">
+        <v>60.3</v>
+      </c>
+      <c r="K69" s="1">
+        <f t="shared" si="4"/>
+        <v>2.8557784079478277E-3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A70" s="1">
+        <v>4</v>
+      </c>
+      <c r="B70" s="1">
+        <v>700</v>
+      </c>
+      <c r="C70" s="1">
+        <v>1</v>
+      </c>
+      <c r="D70" s="1" t="str">
+        <f>A70&amp;"-"&amp;(B70+C70)</f>
+        <v>4-701</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H70" s="1">
+        <v>100</v>
+      </c>
+      <c r="I70" s="1">
+        <v>114</v>
+      </c>
+      <c r="K70" s="1">
+        <f>PI()*(((I70-J70)*10^-3)^2/4)</f>
+        <v>1.0207034531513238E-2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A71" s="1">
+        <v>4</v>
+      </c>
+      <c r="B71" s="1">
+        <v>700</v>
+      </c>
+      <c r="C71" s="1">
+        <v>2</v>
+      </c>
+      <c r="D71" s="1" t="str">
+        <f>A71&amp;"-"&amp;(B71+C71)</f>
+        <v>4-702</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H71" s="1">
+        <v>80</v>
+      </c>
+      <c r="I71" s="1">
+        <v>88.9</v>
+      </c>
+      <c r="K71" s="1">
+        <f>PI()*(((I71-J71)*10^-3)^2/4)</f>
+        <v>6.2071666189443481E-3</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:M1" xr:uid="{80D9219E-119C-467C-9531-507D24E0A5C1}">

</xml_diff>

<commit_message>
s'han afegit els progames per fer el sankey
</commit_message>
<xml_diff>
--- a/docs/punts-mesura.xlsx
+++ b/docs/punts-mesura.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\supersonic-at\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\sxs\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13A5D360-EFC0-4705-99B0-8BCB993DD464}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8723CCF-5F97-4297-8D2B-071211DEE167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{4CA701B3-5EB8-45D8-B6BB-1F057196BE44}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="97">
   <si>
     <t>id</t>
   </si>
@@ -290,15 +290,6 @@
     <t>LI671</t>
   </si>
   <si>
-    <t>id_letter</t>
-  </si>
-  <si>
-    <t>plant_number</t>
-  </si>
-  <si>
-    <t>measure_number</t>
-  </si>
-  <si>
     <t>BV</t>
   </si>
   <si>
@@ -324,6 +315,21 @@
   </si>
   <si>
     <t>EI701</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>y</t>
+  </si>
+  <si>
+    <t>id_aux_1</t>
+  </si>
+  <si>
+    <t>id_aux_2</t>
+  </si>
+  <si>
+    <t>id_aux_3</t>
   </si>
 </sst>
 </file>
@@ -704,7 +710,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80D9219E-119C-467C-9531-507D24E0A5C1}">
-  <dimension ref="A1:K71"/>
+  <dimension ref="A1:M71"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
@@ -717,15 +723,15 @@
     <col min="12" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
@@ -751,10 +757,16 @@
       <c r="K1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1">
         <v>7</v>
@@ -782,10 +794,16 @@
         <f t="shared" ref="K2:K21" si="0">PI()*(((I2-J2)*10^-3)^2/4)</f>
         <v>9.4896329995100878E-2</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L2" s="1">
+        <v>20</v>
+      </c>
+      <c r="M2" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B3" s="1">
         <v>104</v>
@@ -819,10 +837,16 @@
         <f t="shared" si="0"/>
         <v>2.0995460053481439E-2</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L3" s="1">
+        <v>10</v>
+      </c>
+      <c r="M3" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B4" s="1">
         <v>105</v>
@@ -856,10 +880,16 @@
         <f t="shared" si="0"/>
         <v>2.0995460053481439E-2</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L4" s="1">
+        <v>539</v>
+      </c>
+      <c r="M4" s="1">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B5" s="1">
         <v>106</v>
@@ -893,10 +923,16 @@
         <f t="shared" si="0"/>
         <v>2.0995460053481439E-2</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L5" s="1">
+        <v>537</v>
+      </c>
+      <c r="M5" s="1">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B6" s="1">
         <v>107</v>
@@ -930,10 +966,16 @@
         <f t="shared" si="0"/>
         <v>2.0995460053481439E-2</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L6" s="1">
+        <v>692</v>
+      </c>
+      <c r="M6" s="1">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B7" s="1">
         <v>108</v>
@@ -967,10 +1009,16 @@
         <f t="shared" si="0"/>
         <v>2.0995460053481439E-2</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L7" s="1">
+        <v>766</v>
+      </c>
+      <c r="M7" s="1">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B8" s="1">
         <v>109</v>
@@ -1004,8 +1052,14 @@
         <f t="shared" si="0"/>
         <v>3.116510177843532E-2</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L8" s="1">
+        <v>694</v>
+      </c>
+      <c r="M8" s="1">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>1</v>
       </c>
@@ -1036,7 +1090,7 @@
         <v>3.8013271108436497E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>1</v>
       </c>
@@ -1070,7 +1124,7 @@
         <v>1.5614500886504672E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>1</v>
       </c>
@@ -1104,7 +1158,7 @@
         <v>6.2071666189443481E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>1</v>
       </c>
@@ -1138,7 +1192,7 @@
         <v>6.2071666189443481E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>1</v>
       </c>
@@ -1172,7 +1226,7 @@
         <v>3.8013271108436497E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>1</v>
       </c>
@@ -1206,7 +1260,7 @@
         <v>2.8557784079478277E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>1</v>
       </c>
@@ -1240,7 +1294,7 @@
         <v>2.8557784079478277E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>1</v>
       </c>
@@ -2601,7 +2655,7 @@
         <v>2-701</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="H63" s="1">
         <v>150</v>
@@ -2629,7 +2683,7 @@
         <v>2-702</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="H64" s="1">
         <v>100</v>
@@ -2657,7 +2711,7 @@
         <v>2-703</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="H65" s="1">
         <v>100</v>
@@ -2685,7 +2739,7 @@
         <v>2-704</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="H66" s="1">
         <v>65</v>
@@ -2713,7 +2767,7 @@
         <v>2-705</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="H67" s="1">
         <v>50</v>
@@ -2741,7 +2795,7 @@
         <v>2-706</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="H68" s="1">
         <v>65</v>
@@ -2769,7 +2823,7 @@
         <v>2-707</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="H69" s="1">
         <v>50</v>
@@ -2797,7 +2851,7 @@
         <v>4-701</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H70" s="1">
         <v>100</v>
@@ -2825,7 +2879,7 @@
         <v>4-702</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H71" s="1">
         <v>80</v>

</xml_diff>

<commit_message>
abans de fer canvis en el create_plots per dividirlo en funcions mes simples
</commit_message>
<xml_diff>
--- a/docs/punts-mesura.xlsx
+++ b/docs/punts-mesura.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\sxs\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8723CCF-5F97-4297-8D2B-071211DEE167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{684AE619-C271-4304-90E6-60E320674E91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{4CA701B3-5EB8-45D8-B6BB-1F057196BE44}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="96">
   <si>
     <t>id</t>
   </si>
@@ -288,9 +288,6 @@
   </si>
   <si>
     <t>LI671</t>
-  </si>
-  <si>
-    <t>BV</t>
   </si>
   <si>
     <t>VI710</t>
@@ -725,13 +722,13 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>95</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>96</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
@@ -758,305 +755,245 @@
         <v>4</v>
       </c>
       <c r="L1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>93</v>
-      </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>83</v>
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1">
+        <v>100</v>
       </c>
       <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="str">
+        <f>A2&amp;"-"&amp;(B2+C2)</f>
+        <v>1-101</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" s="1">
+        <v>200</v>
+      </c>
+      <c r="I2" s="1">
+        <v>220</v>
+      </c>
+      <c r="K2" s="1">
+        <f>PI()*(((I2-J2)*10^-3)^2/4)</f>
+        <v>3.8013271108436497E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1">
+        <v>100</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1" t="str">
+        <f>A3&amp;"-"&amp;(B3+C3)</f>
+        <v>1-102</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" s="1">
+        <v>125</v>
+      </c>
+      <c r="I3" s="1">
+        <v>141</v>
+      </c>
+      <c r="K3" s="1">
+        <f>PI()*(((I3-J3)*10^-3)^2/4)</f>
+        <v>1.5614500886504672E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>1</v>
+      </c>
+      <c r="B4" s="1">
+        <v>100</v>
+      </c>
+      <c r="C4" s="1">
+        <v>3</v>
+      </c>
+      <c r="D4" s="1" t="str">
+        <f>A4&amp;"-"&amp;(B4+C4)</f>
+        <v>1-103</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="1" t="str">
-        <f>A2&amp;(B2+C2)</f>
-        <v>BV7</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H2" s="1">
-        <v>350</v>
-      </c>
-      <c r="I2" s="1">
-        <v>355.6</v>
-      </c>
-      <c r="J2" s="1">
+      <c r="H4" s="1">
+        <v>80</v>
+      </c>
+      <c r="I4" s="1">
+        <v>88.9</v>
+      </c>
+      <c r="K4" s="1">
+        <f>PI()*(((I4-J4)*10^-3)^2/4)</f>
+        <v>6.2071666189443481E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>1</v>
+      </c>
+      <c r="B5" s="1">
+        <v>100</v>
+      </c>
+      <c r="C5" s="1">
+        <v>4</v>
+      </c>
+      <c r="D5" s="1" t="str">
+        <f>A5&amp;"-"&amp;(B5+C5)</f>
+        <v>1-104</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="1">
-        <f t="shared" ref="K2:K21" si="0">PI()*(((I2-J2)*10^-3)^2/4)</f>
-        <v>9.4896329995100878E-2</v>
-      </c>
-      <c r="L2" s="1">
-        <v>20</v>
-      </c>
-      <c r="M2" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B3" s="1">
-        <v>104</v>
-      </c>
-      <c r="C3" s="1">
+      <c r="H5" s="1">
+        <v>80</v>
+      </c>
+      <c r="I5" s="1">
+        <v>88.9</v>
+      </c>
+      <c r="K5" s="1">
+        <f>PI()*(((I5-J5)*10^-3)^2/4)</f>
+        <v>6.2071666189443481E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>1</v>
+      </c>
+      <c r="B6" s="1">
+        <v>100</v>
+      </c>
+      <c r="C6" s="1">
         <v>5</v>
       </c>
-      <c r="D3" s="1" t="str">
-        <f t="shared" ref="D3:D8" si="1">A3&amp;B3&amp;"-"&amp;C3</f>
-        <v>BV104-5</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H3" s="1">
-        <v>150</v>
-      </c>
-      <c r="I3" s="1">
-        <v>168.3</v>
-      </c>
-      <c r="J3" s="1">
-        <v>4.8</v>
-      </c>
-      <c r="K3" s="1">
-        <f t="shared" si="0"/>
-        <v>2.0995460053481439E-2</v>
-      </c>
-      <c r="L3" s="1">
+      <c r="D6" s="1" t="str">
+        <f>A6&amp;"-"&amp;(B6+C6)</f>
+        <v>1-105</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H6" s="1">
+        <v>200</v>
+      </c>
+      <c r="I6" s="1">
+        <v>220</v>
+      </c>
+      <c r="K6" s="1">
+        <f>PI()*(((I6-J6)*10^-3)^2/4)</f>
+        <v>3.8013271108436497E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>1</v>
+      </c>
+      <c r="B7" s="1">
+        <v>100</v>
+      </c>
+      <c r="C7" s="1">
+        <v>6</v>
+      </c>
+      <c r="D7" s="1" t="str">
+        <f>A7&amp;"-"&amp;(B7+C7)</f>
+        <v>1-106</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="M3" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B4" s="1">
-        <v>105</v>
-      </c>
-      <c r="C4" s="1">
-        <v>1</v>
-      </c>
-      <c r="D4" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>BV105-1</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" s="1">
-        <v>150</v>
-      </c>
-      <c r="I4" s="1">
-        <v>168.3</v>
-      </c>
-      <c r="J4" s="1">
-        <v>4.8</v>
-      </c>
-      <c r="K4" s="1">
-        <f t="shared" si="0"/>
-        <v>2.0995460053481439E-2</v>
-      </c>
-      <c r="L4" s="1">
-        <v>539</v>
-      </c>
-      <c r="M4" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B5" s="1">
-        <v>106</v>
-      </c>
-      <c r="C5" s="1">
-        <v>3</v>
-      </c>
-      <c r="D5" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>BV106-3</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H5" s="1">
-        <v>150</v>
-      </c>
-      <c r="I5" s="1">
-        <v>168.3</v>
-      </c>
-      <c r="J5" s="1">
-        <v>4.8</v>
-      </c>
-      <c r="K5" s="1">
-        <f t="shared" si="0"/>
-        <v>2.0995460053481439E-2</v>
-      </c>
-      <c r="L5" s="1">
-        <v>537</v>
-      </c>
-      <c r="M5" s="1">
-        <v>821</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B6" s="1">
-        <v>107</v>
-      </c>
-      <c r="C6" s="1">
-        <v>2</v>
-      </c>
-      <c r="D6" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>BV107-2</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H6" s="1">
-        <v>150</v>
-      </c>
-      <c r="I6" s="1">
-        <v>168.3</v>
-      </c>
-      <c r="J6" s="1">
-        <v>4.8</v>
-      </c>
-      <c r="K6" s="1">
-        <f t="shared" si="0"/>
-        <v>2.0995460053481439E-2</v>
-      </c>
-      <c r="L6" s="1">
-        <v>692</v>
-      </c>
-      <c r="M6" s="1">
-        <v>709</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B7" s="1">
-        <v>108</v>
-      </c>
-      <c r="C7" s="1">
-        <v>4</v>
-      </c>
-      <c r="D7" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>BV108-4</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>26</v>
-      </c>
       <c r="H7" s="1">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="I7" s="1">
-        <v>168.3</v>
-      </c>
-      <c r="J7" s="1">
-        <v>4.8</v>
+        <v>60.3</v>
       </c>
       <c r="K7" s="1">
-        <f t="shared" si="0"/>
-        <v>2.0995460053481439E-2</v>
-      </c>
-      <c r="L7" s="1">
-        <v>766</v>
-      </c>
-      <c r="M7" s="1">
-        <v>770</v>
+        <f>PI()*(((I7-J7)*10^-3)^2/4)</f>
+        <v>2.8557784079478277E-3</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>83</v>
+      <c r="A8" s="1">
+        <v>1</v>
       </c>
       <c r="B8" s="1">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="C8" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D8" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>BV109-6</v>
+        <f>A8&amp;"-"&amp;(B8+C8)</f>
+        <v>1-107</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="H8" s="1">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="I8" s="1">
-        <v>204</v>
-      </c>
-      <c r="J8" s="1">
-        <v>4.8</v>
+        <v>60.3</v>
       </c>
       <c r="K8" s="1">
-        <f t="shared" si="0"/>
-        <v>3.116510177843532E-2</v>
-      </c>
-      <c r="L8" s="1">
-        <v>694</v>
-      </c>
-      <c r="M8" s="1">
-        <v>829</v>
+        <f>PI()*(((I8-J8)*10^-3)^2/4)</f>
+        <v>2.8557784079478277E-3</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
@@ -1067,27 +1004,27 @@
         <v>100</v>
       </c>
       <c r="C9" s="1">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D9" s="1" t="str">
         <f>A9&amp;"-"&amp;(B9+C9)</f>
-        <v>1-101</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>29</v>
+        <v>1-108</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>7</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H9" s="1">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="I9" s="1">
-        <v>220</v>
+        <v>88.9</v>
       </c>
       <c r="K9" s="1">
-        <f t="shared" si="0"/>
-        <v>3.8013271108436497E-2</v>
+        <f>PI()*(((I9-J9)*10^-3)^2/4)</f>
+        <v>6.2071666189443481E-3</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
@@ -1095,33 +1032,27 @@
         <v>1</v>
       </c>
       <c r="B10" s="1">
-        <v>100</v>
+        <v>700</v>
       </c>
       <c r="C10" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" s="1" t="str">
-        <f t="shared" ref="D10:D69" si="2">A10&amp;"-"&amp;(B10+C10)</f>
-        <v>1-102</v>
+        <f>A10&amp;"-"&amp;(B10+C10)</f>
+        <v>1-701</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="H10" s="1">
-        <v>125</v>
+        <v>200</v>
       </c>
       <c r="I10" s="1">
-        <v>141</v>
+        <v>220</v>
       </c>
       <c r="K10" s="1">
-        <f t="shared" si="0"/>
-        <v>1.5614500886504672E-2</v>
+        <f>PI()*(((I10-J10)*10^-3)^2/4)</f>
+        <v>3.8013271108436497E-2</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
@@ -1129,23 +1060,17 @@
         <v>1</v>
       </c>
       <c r="B11" s="1">
-        <v>100</v>
+        <v>700</v>
       </c>
       <c r="C11" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D11" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-103</v>
+        <f>A11&amp;"-"&amp;(B11+C11)</f>
+        <v>1-702</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>7</v>
+        <v>54</v>
       </c>
       <c r="H11" s="1">
         <v>80</v>
@@ -1154,7 +1079,7 @@
         <v>88.9</v>
       </c>
       <c r="K11" s="1">
-        <f t="shared" si="0"/>
+        <f>PI()*(((I11-J11)*10^-3)^2/4)</f>
         <v>6.2071666189443481E-3</v>
       </c>
     </row>
@@ -1163,33 +1088,21 @@
         <v>1</v>
       </c>
       <c r="B12" s="1">
-        <v>100</v>
+        <v>700</v>
       </c>
       <c r="C12" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D12" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-104</v>
+        <f>A12&amp;"-"&amp;(B12+C12)</f>
+        <v>1-703</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H12" s="1">
-        <v>80</v>
-      </c>
-      <c r="I12" s="1">
-        <v>88.9</v>
+        <v>55</v>
       </c>
       <c r="K12" s="1">
-        <f t="shared" si="0"/>
-        <v>6.2071666189443481E-3</v>
+        <f>PI()*(((I12-J12)*10^-3)^2/4)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
@@ -1197,33 +1110,21 @@
         <v>1</v>
       </c>
       <c r="B13" s="1">
-        <v>100</v>
+        <v>700</v>
       </c>
       <c r="C13" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D13" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-105</v>
+        <f>A13&amp;"-"&amp;(B13+C13)</f>
+        <v>1-704</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="H13" s="1">
-        <v>200</v>
-      </c>
-      <c r="I13" s="1">
-        <v>220</v>
+        <v>56</v>
       </c>
       <c r="K13" s="1">
-        <f t="shared" si="0"/>
-        <v>3.8013271108436497E-2</v>
+        <f>PI()*(((I13-J13)*10^-3)^2/4)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
@@ -1231,33 +1132,27 @@
         <v>1</v>
       </c>
       <c r="B14" s="1">
+        <v>700</v>
+      </c>
+      <c r="C14" s="1">
+        <v>5</v>
+      </c>
+      <c r="D14" s="1" t="str">
+        <f>A14&amp;"-"&amp;(B14+C14)</f>
+        <v>1-705</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="H14" s="1">
         <v>100</v>
       </c>
-      <c r="C14" s="1">
-        <v>6</v>
-      </c>
-      <c r="D14" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-106</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H14" s="1">
-        <v>50</v>
-      </c>
       <c r="I14" s="1">
-        <v>60.3</v>
+        <v>114</v>
       </c>
       <c r="K14" s="1">
-        <f t="shared" si="0"/>
-        <v>2.8557784079478277E-3</v>
+        <f>PI()*(((I14-J14)*10^-3)^2/4)</f>
+        <v>1.0207034531513238E-2</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
@@ -1265,33 +1160,27 @@
         <v>1</v>
       </c>
       <c r="B15" s="1">
-        <v>100</v>
+        <v>700</v>
       </c>
       <c r="C15" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D15" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-107</v>
+        <f>A15&amp;"-"&amp;(B15+C15)</f>
+        <v>1-706</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>11</v>
+        <v>58</v>
       </c>
       <c r="H15" s="1">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="I15" s="1">
-        <v>60.3</v>
+        <v>76.099999999999994</v>
       </c>
       <c r="K15" s="1">
-        <f t="shared" si="0"/>
-        <v>2.8557784079478277E-3</v>
+        <f>PI()*(((I15-J15)*10^-3)^2/4)</f>
+        <v>4.5484056978489359E-3</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
@@ -1299,20 +1188,17 @@
         <v>1</v>
       </c>
       <c r="B16" s="1">
-        <v>100</v>
+        <v>700</v>
       </c>
       <c r="C16" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D16" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-108</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>8</v>
+        <f>A16&amp;"-"&amp;(B16+C16)</f>
+        <v>1-707</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="H16" s="1">
         <v>80</v>
@@ -1321,482 +1207,449 @@
         <v>88.9</v>
       </c>
       <c r="K16" s="1">
-        <f t="shared" si="0"/>
+        <f>PI()*(((I16-J16)*10^-3)^2/4)</f>
         <v>6.2071666189443481E-3</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B17" s="1">
-        <v>100</v>
+        <v>700</v>
       </c>
       <c r="C17" s="1">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D17" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>6-101</v>
+        <f>A17&amp;"-"&amp;(B17+C17)</f>
+        <v>1-708</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H17" s="1">
-        <v>204</v>
+        <v>125</v>
       </c>
       <c r="I17" s="1">
-        <v>204</v>
+        <v>141</v>
       </c>
       <c r="K17" s="1">
-        <f t="shared" si="0"/>
-        <v>3.2685129967948215E-2</v>
+        <f>PI()*(((I17-J17)*10^-3)^2/4)</f>
+        <v>1.5614500886504672E-2</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B18" s="1">
-        <v>100</v>
+        <v>800</v>
       </c>
       <c r="C18" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>6-102</v>
+        <f>A18&amp;"-"&amp;(B18+C18)</f>
+        <v>1-801</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="H18" s="1">
-        <v>204</v>
+        <v>155</v>
       </c>
       <c r="I18" s="1">
-        <v>204</v>
+        <v>155</v>
+      </c>
+      <c r="J18" s="1">
+        <v>1.8</v>
       </c>
       <c r="K18" s="1">
-        <f t="shared" si="0"/>
-        <v>3.2685129967948215E-2</v>
+        <f>PI()*(((I18-J18)*10^-3)^2/4)</f>
+        <v>1.8433483390497326E-2</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B19" s="1">
-        <v>100</v>
+        <v>800</v>
       </c>
       <c r="C19" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D19" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>6-103</v>
+        <f>A19&amp;"-"&amp;(B19+C19)</f>
+        <v>1-802</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="H19" s="1">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="I19" s="1">
-        <v>114</v>
+        <v>88.9</v>
       </c>
       <c r="K19" s="1">
-        <f t="shared" si="0"/>
-        <v>1.0207034531513238E-2</v>
+        <f>PI()*(((I19-J19)*10^-3)^2/4)</f>
+        <v>6.2071666189443481E-3</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B20" s="1">
-        <v>100</v>
+        <v>800</v>
       </c>
       <c r="C20" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D20" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>6-104</v>
+        <f>A20&amp;"-"&amp;(B20+C20)</f>
+        <v>1-803</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="H20" s="1">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="I20" s="1">
-        <v>129</v>
+        <v>139.69999999999999</v>
       </c>
       <c r="K20" s="1">
-        <f t="shared" si="0"/>
-        <v>1.3069810837096936E-2</v>
+        <f>PI()*(((I20-J20)*10^-3)^2/4)</f>
+        <v>1.5327901242699303E-2</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B21" s="1">
-        <v>100</v>
+        <v>900</v>
       </c>
       <c r="C21" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D21" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>6-105</v>
+        <f>A21&amp;"-"&amp;(B21+C21)</f>
+        <v>1-901</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="H21" s="1">
-        <v>129</v>
+        <v>204</v>
       </c>
       <c r="I21" s="1">
-        <v>129</v>
+        <v>204</v>
       </c>
       <c r="K21" s="1">
-        <f t="shared" si="0"/>
-        <v>1.3069810837096936E-2</v>
+        <f>PI()*(((I21-J21)*10^-3)^2/4)</f>
+        <v>3.2685129967948215E-2</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B22" s="1">
-        <v>200</v>
+        <v>900</v>
       </c>
       <c r="C22" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>3-201</v>
+        <f>A22&amp;"-"&amp;(B22+C22)</f>
+        <v>1-902</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="H22" s="1">
-        <v>100</v>
+        <v>204</v>
       </c>
       <c r="I22" s="1">
-        <v>114</v>
+        <v>204</v>
       </c>
       <c r="K22" s="1">
-        <f t="shared" ref="K22:K62" si="3">PI()*(((I22-J22)*10^-3)^2/4)</f>
-        <v>1.0207034531513238E-2</v>
+        <f>PI()*(((I22-J22)*10^-3)^2/4)</f>
+        <v>3.2685129967948215E-2</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
+        <v>1</v>
+      </c>
+      <c r="B23" s="1">
+        <v>900</v>
+      </c>
+      <c r="C23" s="1">
         <v>3</v>
       </c>
-      <c r="B23" s="1">
-        <v>200</v>
-      </c>
-      <c r="C23" s="1">
-        <v>2</v>
-      </c>
       <c r="D23" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>3-202</v>
+        <f>A23&amp;"-"&amp;(B23+C23)</f>
+        <v>1-903</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>38</v>
+        <v>65</v>
       </c>
       <c r="H23" s="1">
-        <v>65</v>
+        <v>204</v>
       </c>
       <c r="I23" s="1">
-        <v>76.099999999999994</v>
+        <v>204</v>
       </c>
       <c r="K23" s="1">
-        <f t="shared" si="3"/>
-        <v>4.5484056978489359E-3</v>
+        <f>PI()*(((I23-J23)*10^-3)^2/4)</f>
+        <v>3.2685129967948215E-2</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B24" s="1">
-        <v>200</v>
+        <v>900</v>
       </c>
       <c r="C24" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D24" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>3-203</v>
+        <f>A24&amp;"-"&amp;(B24+C24)</f>
+        <v>1-904</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>39</v>
+        <v>65</v>
       </c>
       <c r="H24" s="1">
-        <v>65</v>
+        <v>155</v>
       </c>
       <c r="I24" s="1">
-        <v>76.099999999999994</v>
+        <v>154</v>
       </c>
       <c r="K24" s="1">
-        <f t="shared" si="3"/>
-        <v>4.5484056978489359E-3</v>
+        <f>PI()*(((I24-J24)*10^-3)^2/4)</f>
+        <v>1.8626502843133885E-2</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B25" s="1">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="C25" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D25" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>3-301</v>
+        <f>A25&amp;"-"&amp;(B25+C25)</f>
+        <v>1-905</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="H25" s="1">
-        <v>65</v>
+        <v>155</v>
       </c>
       <c r="I25" s="1">
-        <v>76.099999999999994</v>
+        <v>154</v>
       </c>
       <c r="K25" s="1">
-        <f t="shared" si="3"/>
-        <v>4.5484056978489359E-3</v>
+        <f>PI()*(((I25-J25)*10^-3)^2/4)</f>
+        <v>1.8626502843133885E-2</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B26" s="1">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="C26" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D26" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>3-302</v>
+        <f>A26&amp;"-"&amp;(B26+C26)</f>
+        <v>1-906</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="H26" s="1">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="I26" s="1">
-        <v>60.3</v>
+        <v>88.9</v>
       </c>
       <c r="K26" s="1">
-        <f t="shared" si="3"/>
-        <v>2.8557784079478277E-3</v>
+        <f>PI()*(((I26-J26)*10^-3)^2/4)</f>
+        <v>6.2071666189443481E-3</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B27" s="1">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="C27" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D27" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>3-303</v>
+        <f>A27&amp;"-"&amp;(B27+C27)</f>
+        <v>1-907</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="H27" s="1">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="I27" s="1">
-        <v>60.3</v>
+        <v>88.9</v>
       </c>
       <c r="K27" s="1">
-        <f t="shared" si="3"/>
-        <v>2.8557784079478277E-3</v>
+        <f>PI()*(((I27-J27)*10^-3)^2/4)</f>
+        <v>6.2071666189443481E-3</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B28" s="1">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="C28" s="1">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D28" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>3-304</v>
+        <f>A28&amp;"-"&amp;(B28+C28)</f>
+        <v>1-908</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>42</v>
+        <v>70</v>
       </c>
       <c r="H28" s="1">
-        <v>32</v>
+        <v>125</v>
       </c>
       <c r="I28" s="1">
-        <v>42.2</v>
+        <v>139.69999999999999</v>
       </c>
       <c r="K28" s="1">
-        <f t="shared" si="3"/>
-        <v>1.3986684653047119E-3</v>
+        <f>PI()*(((I28-J28)*10^-3)^2/4)</f>
+        <v>1.5327901242699303E-2</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B29" s="1">
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="C29" s="1">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D29" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>3-401</v>
+        <f>A29&amp;"-"&amp;(B29+C29)</f>
+        <v>1-909</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>46</v>
+        <v>71</v>
       </c>
       <c r="H29" s="1">
-        <v>80</v>
+        <v>125</v>
       </c>
       <c r="I29" s="1">
-        <v>88.9</v>
+        <v>139.69999999999999</v>
       </c>
       <c r="K29" s="1">
-        <f t="shared" si="3"/>
-        <v>6.2071666189443481E-3</v>
+        <f>PI()*(((I29-J29)*10^-3)^2/4)</f>
+        <v>1.5327901242699303E-2</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B30" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="C30" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D30" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>3-402</v>
+        <f>A30&amp;"-"&amp;(B30+C30)</f>
+        <v>2-601</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>47</v>
+        <v>77</v>
       </c>
       <c r="H30" s="1">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="I30" s="1">
-        <v>48.3</v>
+        <v>76.099999999999994</v>
       </c>
       <c r="K30" s="1">
-        <f t="shared" si="3"/>
-        <v>1.8322475214082729E-3</v>
+        <f>PI()*(((I30-J30)*10^-3)^2/4)</f>
+        <v>4.5484056978489359E-3</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B31" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="C31" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D31" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>3-403</v>
+        <f>A31&amp;"-"&amp;(B31+C31)</f>
+        <v>2-602</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>48</v>
+        <v>78</v>
       </c>
       <c r="H31" s="1">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="I31" s="1">
-        <v>60.3</v>
+        <v>43</v>
       </c>
       <c r="K31" s="1">
-        <f t="shared" si="3"/>
-        <v>2.8557784079478277E-3</v>
+        <f>PI()*(((I31-J31)*10^-3)^2/4)</f>
+        <v>1.4522012041218821E-3</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
+        <v>2</v>
+      </c>
+      <c r="B32" s="1">
+        <v>600</v>
+      </c>
+      <c r="C32" s="1">
         <v>3</v>
       </c>
-      <c r="B32" s="1">
-        <v>400</v>
-      </c>
-      <c r="C32" s="1">
-        <v>4</v>
-      </c>
       <c r="D32" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>3-404</v>
+        <f>A32&amp;"-"&amp;(B32+C32)</f>
+        <v>2-603</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>49</v>
+        <v>79</v>
       </c>
       <c r="H32" s="1">
         <v>50</v>
@@ -1805,36 +1658,36 @@
         <v>60.3</v>
       </c>
       <c r="K32" s="1">
-        <f t="shared" si="3"/>
+        <f>PI()*(((I32-J32)*10^-3)^2/4)</f>
         <v>2.8557784079478277E-3</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B33" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="C33" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D33" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>3-405</v>
+        <f>A33&amp;"-"&amp;(B33+C33)</f>
+        <v>2-604</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="H33" s="1">
-        <v>40</v>
+        <v>125</v>
       </c>
       <c r="I33" s="1">
-        <v>48.3</v>
+        <v>139</v>
       </c>
       <c r="K33" s="1">
-        <f t="shared" si="3"/>
-        <v>1.8322475214082729E-3</v>
+        <f>PI()*(((I33-J33)*10^-3)^2/4)</f>
+        <v>1.5174677915002103E-2</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.3">
@@ -1845,24 +1698,24 @@
         <v>600</v>
       </c>
       <c r="C34" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D34" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>2-601</v>
+        <f>A34&amp;"-"&amp;(B34+C34)</f>
+        <v>2-605</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="H34" s="1">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="I34" s="1">
-        <v>76.099999999999994</v>
+        <v>114</v>
       </c>
       <c r="K34" s="1">
-        <f t="shared" si="3"/>
-        <v>4.5484056978489359E-3</v>
+        <f>PI()*(((I34-J34)*10^-3)^2/4)</f>
+        <v>1.0207034531513238E-2</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.3">
@@ -1873,24 +1726,24 @@
         <v>600</v>
       </c>
       <c r="C35" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D35" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>2-602</v>
+        <f>A35&amp;"-"&amp;(B35+C35)</f>
+        <v>2-606</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H35" s="1">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="I35" s="1">
-        <v>43</v>
+        <v>60.3</v>
       </c>
       <c r="K35" s="1">
-        <f t="shared" si="3"/>
-        <v>1.4522012041218821E-3</v>
+        <f>PI()*(((I35-J35)*10^-3)^2/4)</f>
+        <v>2.8557784079478277E-3</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.3">
@@ -1898,27 +1751,27 @@
         <v>2</v>
       </c>
       <c r="B36" s="1">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="C36" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D36" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>2-603</v>
+        <f>A36&amp;"-"&amp;(B36+C36)</f>
+        <v>2-701</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="H36" s="1">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="I36" s="1">
-        <v>60.3</v>
+        <v>168.3</v>
       </c>
       <c r="K36" s="1">
-        <f t="shared" si="3"/>
-        <v>2.8557784079478277E-3</v>
+        <f>PI()*(((I36-J36)*10^-3)^2/4)</f>
+        <v>2.2246316584434749E-2</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.3">
@@ -1926,27 +1779,27 @@
         <v>2</v>
       </c>
       <c r="B37" s="1">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="C37" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D37" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>2-604</v>
+        <f>A37&amp;"-"&amp;(B37+C37)</f>
+        <v>2-702</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="H37" s="1">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="I37" s="1">
-        <v>139</v>
+        <v>114</v>
       </c>
       <c r="K37" s="1">
-        <f t="shared" si="3"/>
-        <v>1.5174677915002103E-2</v>
+        <f>PI()*(((I37-J37)*10^-3)^2/4)</f>
+        <v>1.0207034531513238E-2</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
@@ -1954,17 +1807,17 @@
         <v>2</v>
       </c>
       <c r="B38" s="1">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="C38" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D38" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>2-605</v>
+        <f>A38&amp;"-"&amp;(B38+C38)</f>
+        <v>2-703</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="H38" s="1">
         <v>100</v>
@@ -1973,7 +1826,7 @@
         <v>114</v>
       </c>
       <c r="K38" s="1">
-        <f t="shared" si="3"/>
+        <f>PI()*(((I38-J38)*10^-3)^2/4)</f>
         <v>1.0207034531513238E-2</v>
       </c>
     </row>
@@ -1982,45 +1835,45 @@
         <v>2</v>
       </c>
       <c r="B39" s="1">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="C39" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D39" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>2-606</v>
+        <f>A39&amp;"-"&amp;(B39+C39)</f>
+        <v>2-704</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H39" s="1">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="I39" s="1">
-        <v>60.3</v>
+        <v>73</v>
       </c>
       <c r="K39" s="1">
-        <f t="shared" si="3"/>
-        <v>2.8557784079478277E-3</v>
+        <f>PI()*(((I39-J39)*10^-3)^2/4)</f>
+        <v>4.1853868127450016E-3</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B40" s="1">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="C40" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D40" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>3-601</v>
+        <f>A40&amp;"-"&amp;(B40+C40)</f>
+        <v>2-705</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>51</v>
+        <v>84</v>
       </c>
       <c r="H40" s="1">
         <v>50</v>
@@ -2029,54 +1882,54 @@
         <v>60.3</v>
       </c>
       <c r="K40" s="1">
-        <f t="shared" si="3"/>
+        <f>PI()*(((I40-J40)*10^-3)^2/4)</f>
         <v>2.8557784079478277E-3</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B41" s="1">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="C41" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D41" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>3-602</v>
+        <f>A41&amp;"-"&amp;(B41+C41)</f>
+        <v>2-706</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="H41" s="1">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="I41" s="1">
-        <v>60.3</v>
+        <v>76.099999999999994</v>
       </c>
       <c r="K41" s="1">
-        <f t="shared" si="3"/>
-        <v>2.8557784079478277E-3</v>
+        <f>PI()*(((I41-J41)*10^-3)^2/4)</f>
+        <v>4.5484056978489359E-3</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B42" s="1">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="C42" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D42" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>3-603</v>
+        <f>A42&amp;"-"&amp;(B42+C42)</f>
+        <v>2-707</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>53</v>
+        <v>86</v>
       </c>
       <c r="H42" s="1">
         <v>50</v>
@@ -2091,459 +1944,504 @@
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B43" s="1">
-        <v>700</v>
+        <v>200</v>
       </c>
       <c r="C43" s="1">
         <v>1</v>
       </c>
       <c r="D43" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-701</v>
+        <f>A43&amp;"-"&amp;(B43+C43)</f>
+        <v>3-201</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>60</v>
+        <v>35</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>35</v>
       </c>
       <c r="H43" s="1">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="I43" s="1">
-        <v>220</v>
+        <v>114</v>
       </c>
       <c r="K43" s="1">
-        <f t="shared" si="3"/>
-        <v>3.8013271108436497E-2</v>
+        <f>PI()*(((I43-J43)*10^-3)^2/4)</f>
+        <v>1.0207034531513238E-2</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B44" s="1">
-        <v>700</v>
+        <v>200</v>
       </c>
       <c r="C44" s="1">
         <v>2</v>
       </c>
       <c r="D44" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-702</v>
+        <f>A44&amp;"-"&amp;(B44+C44)</f>
+        <v>3-202</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>54</v>
+        <v>36</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>38</v>
       </c>
       <c r="H44" s="1">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="I44" s="1">
-        <v>88.9</v>
+        <v>76.099999999999994</v>
       </c>
       <c r="K44" s="1">
-        <f t="shared" si="3"/>
-        <v>6.2071666189443481E-3</v>
+        <f>PI()*(((I44-J44)*10^-3)^2/4)</f>
+        <v>4.5484056978489359E-3</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B45" s="1">
-        <v>700</v>
+        <v>200</v>
       </c>
       <c r="C45" s="1">
         <v>3</v>
       </c>
       <c r="D45" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-703</v>
+        <f>A45&amp;"-"&amp;(B45+C45)</f>
+        <v>3-203</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>55</v>
+        <v>37</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H45" s="1">
+        <v>65</v>
+      </c>
+      <c r="I45" s="1">
+        <v>76.099999999999994</v>
       </c>
       <c r="K45" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f>PI()*(((I45-J45)*10^-3)^2/4)</f>
+        <v>4.5484056978489359E-3</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B46" s="1">
-        <v>700</v>
+        <v>300</v>
       </c>
       <c r="C46" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D46" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-704</v>
+        <f>A46&amp;"-"&amp;(B46+C46)</f>
+        <v>3-301</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>56</v>
+        <v>43</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H46" s="1">
+        <v>65</v>
+      </c>
+      <c r="I46" s="1">
+        <v>76.099999999999994</v>
       </c>
       <c r="K46" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f>PI()*(((I46-J46)*10^-3)^2/4)</f>
+        <v>4.5484056978489359E-3</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B47" s="1">
-        <v>700</v>
+        <v>300</v>
       </c>
       <c r="C47" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D47" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-705</v>
+        <f>A47&amp;"-"&amp;(B47+C47)</f>
+        <v>3-302</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>57</v>
+        <v>40</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>44</v>
       </c>
       <c r="H47" s="1">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="I47" s="1">
-        <v>114</v>
+        <v>60.3</v>
       </c>
       <c r="K47" s="1">
-        <f t="shared" si="3"/>
-        <v>1.0207034531513238E-2</v>
+        <f>PI()*(((I47-J47)*10^-3)^2/4)</f>
+        <v>2.8557784079478277E-3</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B48" s="1">
-        <v>700</v>
+        <v>300</v>
       </c>
       <c r="C48" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D48" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-706</v>
+        <f>A48&amp;"-"&amp;(B48+C48)</f>
+        <v>3-303</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>58</v>
+        <v>41</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>45</v>
       </c>
       <c r="H48" s="1">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="I48" s="1">
-        <v>76.099999999999994</v>
+        <v>60.3</v>
       </c>
       <c r="K48" s="1">
-        <f t="shared" si="3"/>
-        <v>4.5484056978489359E-3</v>
+        <f>PI()*(((I48-J48)*10^-3)^2/4)</f>
+        <v>2.8557784079478277E-3</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B49" s="1">
-        <v>700</v>
+        <v>300</v>
       </c>
       <c r="C49" s="1">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D49" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-707</v>
+        <f>A49&amp;"-"&amp;(B49+C49)</f>
+        <v>3-304</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>59</v>
+        <v>42</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>42</v>
       </c>
       <c r="H49" s="1">
-        <v>80</v>
+        <v>32</v>
       </c>
       <c r="I49" s="1">
-        <v>88.9</v>
+        <v>42.2</v>
       </c>
       <c r="K49" s="1">
-        <f t="shared" si="3"/>
-        <v>6.2071666189443481E-3</v>
+        <f>PI()*(((I49-J49)*10^-3)^2/4)</f>
+        <v>1.3986684653047119E-3</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B50" s="1">
-        <v>700</v>
+        <v>400</v>
       </c>
       <c r="C50" s="1">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D50" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-708</v>
+        <f>A50&amp;"-"&amp;(B50+C50)</f>
+        <v>3-401</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>73</v>
+        <v>46</v>
       </c>
       <c r="H50" s="1">
-        <v>125</v>
+        <v>80</v>
       </c>
       <c r="I50" s="1">
-        <v>141</v>
+        <v>88.9</v>
       </c>
       <c r="K50" s="1">
-        <f t="shared" si="3"/>
-        <v>1.5614500886504672E-2</v>
+        <f>PI()*(((I50-J50)*10^-3)^2/4)</f>
+        <v>6.2071666189443481E-3</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B51" s="1">
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="C51" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D51" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-801</v>
+        <f>A51&amp;"-"&amp;(B51+C51)</f>
+        <v>3-402</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="H51" s="1">
-        <v>155</v>
+        <v>40</v>
       </c>
       <c r="I51" s="1">
-        <v>155</v>
-      </c>
-      <c r="J51" s="1">
-        <v>1.8</v>
+        <v>48.3</v>
       </c>
       <c r="K51" s="1">
-        <f t="shared" si="3"/>
-        <v>1.8433483390497326E-2</v>
+        <f>PI()*(((I51-J51)*10^-3)^2/4)</f>
+        <v>1.8322475214082729E-3</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A52" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B52" s="1">
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="C52" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D52" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-802</v>
+        <f>A52&amp;"-"&amp;(B52+C52)</f>
+        <v>3-403</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="H52" s="1">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="I52" s="1">
-        <v>88.9</v>
+        <v>60.3</v>
       </c>
       <c r="K52" s="1">
-        <f t="shared" si="3"/>
-        <v>6.2071666189443481E-3</v>
+        <f>PI()*(((I52-J52)*10^-3)^2/4)</f>
+        <v>2.8557784079478277E-3</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B53" s="1">
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="C53" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D53" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-803</v>
+        <f>A53&amp;"-"&amp;(B53+C53)</f>
+        <v>3-404</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="H53" s="1">
-        <v>125</v>
+        <v>50</v>
       </c>
       <c r="I53" s="1">
-        <v>139.69999999999999</v>
+        <v>60.3</v>
       </c>
       <c r="K53" s="1">
-        <f t="shared" si="3"/>
-        <v>1.5327901242699303E-2</v>
+        <f>PI()*(((I53-J53)*10^-3)^2/4)</f>
+        <v>2.8557784079478277E-3</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B54" s="1">
-        <v>900</v>
+        <v>400</v>
       </c>
       <c r="C54" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D54" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-901</v>
+        <f>A54&amp;"-"&amp;(B54+C54)</f>
+        <v>3-405</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="H54" s="1">
-        <v>204</v>
+        <v>40</v>
       </c>
       <c r="I54" s="1">
-        <v>204</v>
+        <v>48.3</v>
       </c>
       <c r="K54" s="1">
-        <f t="shared" si="3"/>
-        <v>3.2685129967948215E-2</v>
+        <f>PI()*(((I54-J54)*10^-3)^2/4)</f>
+        <v>1.8322475214082729E-3</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B55" s="1">
-        <v>900</v>
+        <v>600</v>
       </c>
       <c r="C55" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D55" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-902</v>
+        <f>A55&amp;"-"&amp;(B55+C55)</f>
+        <v>3-601</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="H55" s="1">
-        <v>204</v>
+        <v>50</v>
       </c>
       <c r="I55" s="1">
-        <v>204</v>
+        <v>60.3</v>
       </c>
       <c r="K55" s="1">
-        <f t="shared" si="3"/>
-        <v>3.2685129967948215E-2</v>
+        <f>PI()*(((I55-J55)*10^-3)^2/4)</f>
+        <v>2.8557784079478277E-3</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A56" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B56" s="1">
-        <v>900</v>
+        <v>600</v>
       </c>
       <c r="C56" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D56" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-903</v>
+        <f>A56&amp;"-"&amp;(B56+C56)</f>
+        <v>3-602</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="H56" s="1">
-        <v>204</v>
+        <v>50</v>
       </c>
       <c r="I56" s="1">
-        <v>204</v>
+        <v>60.3</v>
       </c>
       <c r="K56" s="1">
-        <f t="shared" si="3"/>
-        <v>3.2685129967948215E-2</v>
+        <f>PI()*(((I56-J56)*10^-3)^2/4)</f>
+        <v>2.8557784079478277E-3</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A57" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B57" s="1">
-        <v>900</v>
+        <v>600</v>
       </c>
       <c r="C57" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D57" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-904</v>
+        <f>A57&amp;"-"&amp;(B57+C57)</f>
+        <v>3-603</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="H57" s="1">
-        <v>155</v>
+        <v>50</v>
       </c>
       <c r="I57" s="1">
-        <v>154</v>
+        <v>60.3</v>
       </c>
       <c r="K57" s="1">
-        <f t="shared" si="3"/>
-        <v>1.8626502843133885E-2</v>
+        <f>PI()*(((I57-J57)*10^-3)^2/4)</f>
+        <v>2.8557784079478277E-3</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A58" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B58" s="1">
-        <v>900</v>
+        <v>700</v>
       </c>
       <c r="C58" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D58" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-905</v>
+        <f>A58&amp;"-"&amp;(B58+C58)</f>
+        <v>4-701</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="H58" s="1">
-        <v>155</v>
+        <v>100</v>
       </c>
       <c r="I58" s="1">
-        <v>154</v>
+        <v>114</v>
       </c>
       <c r="K58" s="1">
-        <f t="shared" si="3"/>
-        <v>1.8626502843133885E-2</v>
+        <f>PI()*(((I58-J58)*10^-3)^2/4)</f>
+        <v>1.0207034531513238E-2</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A59" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B59" s="1">
-        <v>900</v>
+        <v>700</v>
       </c>
       <c r="C59" s="1">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D59" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-906</v>
+        <f>A59&amp;"-"&amp;(B59+C59)</f>
+        <v>4-702</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="H59" s="1">
         <v>80</v>
@@ -2552,350 +2450,428 @@
         <v>88.9</v>
       </c>
       <c r="K59" s="1">
-        <f t="shared" si="3"/>
+        <f>PI()*(((I59-J59)*10^-3)^2/4)</f>
         <v>6.2071666189443481E-3</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A60" s="1">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B60" s="1">
-        <v>900</v>
+        <v>100</v>
       </c>
       <c r="C60" s="1">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D60" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-907</v>
+        <f>A60&amp;"-"&amp;(B60+C60)</f>
+        <v>6-101</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="H60" s="1">
-        <v>80</v>
+        <v>204</v>
       </c>
       <c r="I60" s="1">
-        <v>88.9</v>
+        <v>204</v>
       </c>
       <c r="K60" s="1">
-        <f t="shared" si="3"/>
-        <v>6.2071666189443481E-3</v>
+        <f>PI()*(((I60-J60)*10^-3)^2/4)</f>
+        <v>3.2685129967948215E-2</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A61" s="1">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B61" s="1">
-        <v>900</v>
+        <v>100</v>
       </c>
       <c r="C61" s="1">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D61" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-908</v>
+        <f>A61&amp;"-"&amp;(B61+C61)</f>
+        <v>6-102</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="H61" s="1">
-        <v>125</v>
+        <v>204</v>
       </c>
       <c r="I61" s="1">
-        <v>139.69999999999999</v>
+        <v>204</v>
       </c>
       <c r="K61" s="1">
-        <f t="shared" si="3"/>
-        <v>1.5327901242699303E-2</v>
+        <f>PI()*(((I61-J61)*10^-3)^2/4)</f>
+        <v>3.2685129967948215E-2</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A62" s="1">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B62" s="1">
-        <v>900</v>
+        <v>100</v>
       </c>
       <c r="C62" s="1">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D62" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>1-909</v>
+        <f>A62&amp;"-"&amp;(B62+C62)</f>
+        <v>6-103</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="H62" s="1">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="I62" s="1">
-        <v>139.69999999999999</v>
+        <v>114</v>
       </c>
       <c r="K62" s="1">
-        <f t="shared" si="3"/>
-        <v>1.5327901242699303E-2</v>
+        <f>PI()*(((I62-J62)*10^-3)^2/4)</f>
+        <v>1.0207034531513238E-2</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A63" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B63" s="1">
-        <v>700</v>
+        <v>100</v>
       </c>
       <c r="C63" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D63" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>2-701</v>
+        <f>A63&amp;"-"&amp;(B63+C63)</f>
+        <v>6-104</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="H63" s="1">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="I63" s="1">
-        <v>168.3</v>
+        <v>129</v>
       </c>
       <c r="K63" s="1">
-        <f t="shared" ref="K63:K69" si="4">PI()*(((I63-J63)*10^-3)^2/4)</f>
-        <v>2.2246316584434749E-2</v>
+        <f>PI()*(((I63-J63)*10^-3)^2/4)</f>
+        <v>1.3069810837096936E-2</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A64" s="1">
+        <v>6</v>
+      </c>
+      <c r="B64" s="1">
+        <v>100</v>
+      </c>
+      <c r="C64" s="1">
+        <v>5</v>
+      </c>
+      <c r="D64" s="1" t="str">
+        <f>A64&amp;"-"&amp;(B64+C64)</f>
+        <v>6-105</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="H64" s="1">
+        <v>129</v>
+      </c>
+      <c r="I64" s="1">
+        <v>129</v>
+      </c>
+      <c r="K64" s="1">
+        <f>PI()*(((I64-J64)*10^-3)^2/4)</f>
+        <v>1.3069810837096936E-2</v>
+      </c>
+    </row>
+    <row r="65" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="C65" s="1">
+        <v>7</v>
+      </c>
+      <c r="D65" s="1" t="str">
+        <f>A65&amp;(B65+C65)</f>
+        <v>7</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H65" s="1">
+        <v>350</v>
+      </c>
+      <c r="I65" s="1">
+        <v>355.6</v>
+      </c>
+      <c r="J65" s="1">
+        <v>8</v>
+      </c>
+      <c r="K65" s="1">
+        <f>PI()*(((I65-J65)*10^-3)^2/4)</f>
+        <v>9.4896329995100878E-2</v>
+      </c>
+      <c r="L65" s="1">
+        <v>20</v>
+      </c>
+      <c r="M65" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="66" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B66" s="1">
+        <v>104</v>
+      </c>
+      <c r="C66" s="1">
+        <v>5</v>
+      </c>
+      <c r="D66" s="1" t="str">
+        <f>C66&amp;"-"&amp;B66</f>
+        <v>5-104</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H66" s="1">
+        <v>150</v>
+      </c>
+      <c r="I66" s="1">
+        <v>168.3</v>
+      </c>
+      <c r="J66" s="1">
+        <v>4.8</v>
+      </c>
+      <c r="K66" s="1">
+        <f>PI()*(((I66-J66)*10^-3)^2/4)</f>
+        <v>2.0995460053481439E-2</v>
+      </c>
+      <c r="L66" s="1">
+        <v>10</v>
+      </c>
+      <c r="M66" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="67" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B67" s="1">
+        <v>105</v>
+      </c>
+      <c r="C67" s="1">
+        <v>1</v>
+      </c>
+      <c r="D67" s="1" t="str">
+        <f>C67&amp;"-"&amp;B67</f>
+        <v>1-105</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H67" s="1">
+        <v>150</v>
+      </c>
+      <c r="I67" s="1">
+        <v>168.3</v>
+      </c>
+      <c r="J67" s="1">
+        <v>4.8</v>
+      </c>
+      <c r="K67" s="1">
+        <f>PI()*(((I67-J67)*10^-3)^2/4)</f>
+        <v>2.0995460053481439E-2</v>
+      </c>
+      <c r="L67" s="1">
+        <v>539</v>
+      </c>
+      <c r="M67" s="1">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="68" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B68" s="1">
+        <v>106</v>
+      </c>
+      <c r="C68" s="1">
+        <v>3</v>
+      </c>
+      <c r="D68" s="1" t="str">
+        <f>C68&amp;"-"&amp;B68</f>
+        <v>3-106</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H68" s="1">
+        <v>150</v>
+      </c>
+      <c r="I68" s="1">
+        <v>168.3</v>
+      </c>
+      <c r="J68" s="1">
+        <v>4.8</v>
+      </c>
+      <c r="K68" s="1">
+        <f>PI()*(((I68-J68)*10^-3)^2/4)</f>
+        <v>2.0995460053481439E-2</v>
+      </c>
+      <c r="L68" s="1">
+        <v>537</v>
+      </c>
+      <c r="M68" s="1">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="69" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B69" s="1">
+        <v>107</v>
+      </c>
+      <c r="C69" s="1">
         <v>2</v>
       </c>
-      <c r="B64" s="1">
-        <v>700</v>
-      </c>
-      <c r="C64" s="1">
-        <v>2</v>
-      </c>
-      <c r="D64" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>2-702</v>
-      </c>
-      <c r="E64" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="H64" s="1">
-        <v>100</v>
-      </c>
-      <c r="I64" s="1">
-        <v>114</v>
-      </c>
-      <c r="K64" s="1">
-        <f t="shared" si="4"/>
-        <v>1.0207034531513238E-2</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A65" s="1">
-        <v>2</v>
-      </c>
-      <c r="B65" s="1">
-        <v>700</v>
-      </c>
-      <c r="C65" s="1">
-        <v>3</v>
-      </c>
-      <c r="D65" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>2-703</v>
-      </c>
-      <c r="E65" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H65" s="1">
-        <v>100</v>
-      </c>
-      <c r="I65" s="1">
-        <v>114</v>
-      </c>
-      <c r="K65" s="1">
-        <f t="shared" si="4"/>
-        <v>1.0207034531513238E-2</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A66" s="1">
-        <v>2</v>
-      </c>
-      <c r="B66" s="1">
-        <v>700</v>
-      </c>
-      <c r="C66" s="1">
+      <c r="D69" s="1" t="str">
+        <f>C69&amp;"-"&amp;B69</f>
+        <v>2-107</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H69" s="1">
+        <v>150</v>
+      </c>
+      <c r="I69" s="1">
+        <v>168.3</v>
+      </c>
+      <c r="J69" s="1">
+        <v>4.8</v>
+      </c>
+      <c r="K69" s="1">
+        <f>PI()*(((I69-J69)*10^-3)^2/4)</f>
+        <v>2.0995460053481439E-2</v>
+      </c>
+      <c r="L69" s="1">
+        <v>692</v>
+      </c>
+      <c r="M69" s="1">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="70" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B70" s="1">
+        <v>108</v>
+      </c>
+      <c r="C70" s="1">
         <v>4</v>
       </c>
-      <c r="D66" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>2-704</v>
-      </c>
-      <c r="E66" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="H66" s="1">
-        <v>65</v>
-      </c>
-      <c r="I66" s="1">
-        <v>73</v>
-      </c>
-      <c r="K66" s="1">
-        <f t="shared" si="4"/>
-        <v>4.1853868127450016E-3</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A67" s="1">
-        <v>2</v>
-      </c>
-      <c r="B67" s="1">
-        <v>700</v>
-      </c>
-      <c r="C67" s="1">
-        <v>5</v>
-      </c>
-      <c r="D67" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>2-705</v>
-      </c>
-      <c r="E67" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="H67" s="1">
-        <v>50</v>
-      </c>
-      <c r="I67" s="1">
-        <v>60.3</v>
-      </c>
-      <c r="K67" s="1">
-        <f t="shared" si="4"/>
-        <v>2.8557784079478277E-3</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A68" s="1">
-        <v>2</v>
-      </c>
-      <c r="B68" s="1">
-        <v>700</v>
-      </c>
-      <c r="C68" s="1">
-        <v>6</v>
-      </c>
-      <c r="D68" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>2-706</v>
-      </c>
-      <c r="E68" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="H68" s="1">
-        <v>65</v>
-      </c>
-      <c r="I68" s="1">
-        <v>76.099999999999994</v>
-      </c>
-      <c r="K68" s="1">
-        <f t="shared" si="4"/>
-        <v>4.5484056978489359E-3</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A69" s="1">
-        <v>2</v>
-      </c>
-      <c r="B69" s="1">
-        <v>700</v>
-      </c>
-      <c r="C69" s="1">
-        <v>7</v>
-      </c>
-      <c r="D69" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>2-707</v>
-      </c>
-      <c r="E69" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="H69" s="1">
-        <v>50</v>
-      </c>
-      <c r="I69" s="1">
-        <v>60.3</v>
-      </c>
-      <c r="K69" s="1">
-        <f t="shared" si="4"/>
-        <v>2.8557784079478277E-3</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A70" s="1">
-        <v>4</v>
-      </c>
-      <c r="B70" s="1">
-        <v>700</v>
-      </c>
-      <c r="C70" s="1">
-        <v>1</v>
-      </c>
       <c r="D70" s="1" t="str">
-        <f>A70&amp;"-"&amp;(B70+C70)</f>
-        <v>4-701</v>
+        <f>C70&amp;"-"&amp;B70</f>
+        <v>4-108</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>91</v>
+        <v>16</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>26</v>
       </c>
       <c r="H70" s="1">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="I70" s="1">
-        <v>114</v>
+        <v>168.3</v>
+      </c>
+      <c r="J70" s="1">
+        <v>4.8</v>
       </c>
       <c r="K70" s="1">
         <f>PI()*(((I70-J70)*10^-3)^2/4)</f>
-        <v>1.0207034531513238E-2</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A71" s="1">
-        <v>4</v>
-      </c>
+        <v>2.0995460053481439E-2</v>
+      </c>
+      <c r="L70" s="1">
+        <v>766</v>
+      </c>
+      <c r="M70" s="1">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="71" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B71" s="1">
-        <v>700</v>
+        <v>109</v>
       </c>
       <c r="C71" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D71" s="1" t="str">
-        <f>A71&amp;"-"&amp;(B71+C71)</f>
-        <v>4-702</v>
+        <f>C71&amp;"-"&amp;B71</f>
+        <v>6-109</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>91</v>
+        <v>18</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G71" s="1" t="s">
+        <v>26</v>
       </c>
       <c r="H71" s="1">
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="I71" s="1">
-        <v>88.9</v>
+        <v>204</v>
+      </c>
+      <c r="J71" s="1">
+        <v>4.8</v>
       </c>
       <c r="K71" s="1">
         <f>PI()*(((I71-J71)*10^-3)^2/4)</f>
-        <v>6.2071666189443481E-3</v>
+        <v>3.116510177843532E-2</v>
+      </c>
+      <c r="L71" s="1">
+        <v>694</v>
+      </c>
+      <c r="M71" s="1">
+        <v>829</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:M1" xr:uid="{80D9219E-119C-467C-9531-507D24E0A5C1}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M63">
-      <sortCondition ref="B1"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M82">
+      <sortCondition ref="A1"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>